<commit_message>
Add MFP Database with Microsfot Access 1. The mfp database is added with Microsoft Access 2007-2016 2. The mfp database has data from the first 3 lines of the MFP Excel    file 3. The mfp database db model is based on the one currently provided
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/MFP-tests.xlsx
+++ b/src/test/resources/testData/MFP-tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rachowdhury\Documents\Software\mtf-automation-testing-api\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D27E98-6FF6-4C34-9BA5-090CF8DDC913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B61F7A-A1BB-4625-BBAD-B9271D9E90EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>test_case_id</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t xml:space="preserve"> select ndc_eleven, effective_date from mfp;</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> getFromFile("ndc_eleven", "effective_date")</t>
   </si>
   <si>
     <t>Test NDC-11 and Effective Date Dynamicly</t>
@@ -80,6 +77,18 @@
 		"effective_date": "1/1/2026"
 	}
 ]</t>
+  </si>
+  <si>
+    <t>Test NDC-11 and Effective Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> getFromFile("NDC-11", "MFP Effective Date")</t>
+  </si>
+  <si>
+    <t>Test NDC-11 and Effective Date Dynamicly No Function needed</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NDC-11, MFP Effective Date</t>
   </si>
 </sst>
 </file>
@@ -563,10 +572,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -923,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultColWidth="20" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
@@ -958,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
         <v>4</v>
@@ -992,18 +1004,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="256.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="5" spans="1:6" s="2" customFormat="1" ht="148.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1011,13 +1023,27 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>